<commit_message>
Updated student import template
</commit_message>
<xml_diff>
--- a/public/documents/template.xlsx
+++ b/public/documents/template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">學校名稱</t>
   </si>
@@ -44,6 +44,40 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">中學</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">重要：請務必依表單欄位提供資料，</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <u val="single"/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">請勿</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">新增、刪除、更改欄位，以免出現上載錯誤。</t>
     </r>
   </si>
   <si>
@@ -165,7 +199,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -210,12 +244,20 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
+    </font>
+    <font>
       <b val="true"/>
+      <u val="single"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
+      <color rgb="FFFF0000"/>
+      <name val="細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
     </font>
     <font>
       <b val="true"/>
@@ -251,12 +293,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -320,11 +368,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -340,6 +384,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -348,7 +396,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -392,8 +440,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3"/>
+    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -403,25 +453,25 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -429,19 +479,19 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>6</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G4" s="8" t="n">
         <v>23456788</v>

</xml_diff>